<commit_message>
Stage 2 [2:1] [1:2]
</commit_message>
<xml_diff>
--- a/file/history.xlsx
+++ b/file/history.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ckkil\Documents\GitHub\ck-tools\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12EFF942-ED6A-422F-B8EA-DF097D994507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AF945DA-A2A1-4EEF-AAE0-318AF0F42255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5400" yWindow="2850" windowWidth="21600" windowHeight="11295" xr2:uid="{39BF18F1-6CA4-42F4-B020-2D59954264FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{39BF18F1-6CA4-42F4-B020-2D59954264FB}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1876" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1961" uniqueCount="163">
   <si>
     <t>Wizards</t>
   </si>
@@ -522,13 +522,16 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>Cache</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -546,6 +549,12 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -583,7 +592,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -596,9 +605,17 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -933,7 +950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECD49EDF-97AD-42E2-9203-75390A90C7F2}">
-  <dimension ref="A1:F375"/>
+  <dimension ref="A1:F392"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" style="1" customWidth="1"/>
@@ -8217,7 +8234,7 @@
       <c r="D364" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E364" s="6" t="s">
+      <c r="E364" s="1" t="s">
         <v>160</v>
       </c>
       <c r="F364" s="3">
@@ -8277,7 +8294,7 @@
       <c r="D367" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E367" s="6" t="s">
+      <c r="E367" s="1" t="s">
         <v>160</v>
       </c>
       <c r="F367" s="3">
@@ -8317,7 +8334,7 @@
       <c r="D369" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E369" s="6" t="s">
+      <c r="E369" s="1" t="s">
         <v>160</v>
       </c>
       <c r="F369" s="3">
@@ -8357,7 +8374,7 @@
       <c r="D371" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E371" s="6" t="s">
+      <c r="E371" s="1" t="s">
         <v>160</v>
       </c>
       <c r="F371" s="3">
@@ -8377,7 +8394,7 @@
       <c r="D372" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E372" s="6" t="s">
+      <c r="E372" s="1" t="s">
         <v>160</v>
       </c>
       <c r="F372" s="3">
@@ -8425,23 +8442,363 @@
       </c>
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A375" s="4" t="s">
+      <c r="A375" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B375" s="4" t="s">
+      <c r="B375" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C375" s="4" t="s">
+      <c r="C375" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D375" s="4" t="s">
+      <c r="D375" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E375" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F375" s="5">
+      <c r="E375" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F375" s="10">
         <v>46102</v>
+      </c>
+    </row>
+    <row r="376" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A376" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B376" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C376" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D376" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E376" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F376" s="8">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="377" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A377" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B377" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C377" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D377" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E377" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F377" s="8">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="378" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A378" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B378" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C378" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D378" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="E378" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F378" s="8">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="379" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A379" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B379" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C379" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D379" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E379" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F379" s="10">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="380" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A380" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B380" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C380" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D380" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E380" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F380" s="10">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="381" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A381" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B381" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C381" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D381" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E381" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F381" s="10">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="382" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A382" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B382" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C382" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D382" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E382" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F382" s="8">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="383" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A383" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B383" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C383" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D383" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E383" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F383" s="8">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="384" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A384" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B384" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C384" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D384" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E384" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F384" s="10">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="385" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A385" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B385" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C385" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D385" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E385" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F385" s="10">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="386" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A386" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B386" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C386" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D386" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E386" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F386" s="10">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="387" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A387" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B387" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C387" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D387" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E387" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F387" s="8">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="388" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A388" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B388" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C388" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D388" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E388" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F388" s="8">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="389" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A389" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B389" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C389" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D389" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E389" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F389" s="8">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="390" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A390" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B390" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C390" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D390" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E390" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F390" s="10">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="391" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A391" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B391" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C391" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D391" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E391" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F391" s="10">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="392" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A392" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B392" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C392" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="D392" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E392" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F392" s="10">
+        <v>46143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Winamax Spanish Circuit 2026 Stage 1
</commit_message>
<xml_diff>
--- a/file/history.xlsx
+++ b/file/history.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Braga\OneDrive\Documentos\GitHub\ck-tools\file\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/faa3f9bfbb5dc780/Documentos/GitHub/ck-tools/file/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB7ADBC0-0AFC-4EB5-BDC6-F57936754D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="199" documentId="13_ncr:1_{AB7ADBC0-0AFC-4EB5-BDC6-F57936754D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAE06C51-1287-4C3D-8F99-72B017C589A6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{39BF18F1-6CA4-42F4-B020-2D59954264FB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2311" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2473" uniqueCount="209">
   <si>
     <t>Team 1</t>
   </si>
@@ -558,6 +558,111 @@
   </si>
   <si>
     <t>Counter Logic</t>
+  </si>
+  <si>
+    <t>MAD Lions</t>
+  </si>
+  <si>
+    <t>Heroic Academy</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2026</t>
+  </si>
+  <si>
+    <t>Fnatic</t>
+  </si>
+  <si>
+    <t>NIP Impact</t>
+  </si>
+  <si>
+    <t>ENCE Academy</t>
+  </si>
+  <si>
+    <t>100 Thieves</t>
+  </si>
+  <si>
+    <t>SKYFURY</t>
+  </si>
+  <si>
+    <t>FlyQuest RED</t>
+  </si>
+  <si>
+    <t>BIG Academy</t>
+  </si>
+  <si>
+    <t>MOUZ NXT</t>
+  </si>
+  <si>
+    <t>QMISTRY</t>
+  </si>
+  <si>
+    <t>mousesports</t>
+  </si>
+  <si>
+    <t>NOVAQ</t>
+  </si>
+  <si>
+    <t>Gambit</t>
+  </si>
+  <si>
+    <t>Wildcard Academy</t>
+  </si>
+  <si>
+    <t>Nordix</t>
+  </si>
+  <si>
+    <t>VeryGames</t>
+  </si>
+  <si>
+    <t>Astralis Talent</t>
+  </si>
+  <si>
+    <t>Astana Dragons</t>
+  </si>
+  <si>
+    <t>Quantum Bellator Fire</t>
+  </si>
+  <si>
+    <t>Copenhagen Wolves</t>
+  </si>
+  <si>
+    <t>00 Nation</t>
+  </si>
+  <si>
+    <t>Misfits</t>
+  </si>
+  <si>
+    <t>ESC</t>
+  </si>
+  <si>
+    <t>Flash</t>
+  </si>
+  <si>
+    <t>Kinguin</t>
+  </si>
+  <si>
+    <t>Vertigo</t>
+  </si>
+  <si>
+    <t>0x13</t>
+  </si>
+  <si>
+    <t>Space Soldiers</t>
+  </si>
+  <si>
+    <t>Fluffy Gangsters</t>
+  </si>
+  <si>
+    <t>HAVU</t>
+  </si>
+  <si>
+    <t>Movistar KOI</t>
+  </si>
+  <si>
+    <t>GhoulsW</t>
+  </si>
+  <si>
+    <t>Vox Eminor</t>
   </si>
 </sst>
 </file>
@@ -665,10 +770,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -687,7 +792,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1003,14 +1108,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECD49EDF-97AD-42E2-9203-75390A90C7F2}">
-  <dimension ref="A1:G463"/>
+  <dimension ref="A1:H519"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="16.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="39.7109375" customWidth="1"/>
+    <col min="5" max="5" width="39.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.42578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9911,7 +10016,7 @@
       <c r="D445" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E445" s="12" t="s">
+      <c r="E445" s="4" t="s">
         <v>164</v>
       </c>
       <c r="F445" s="9">
@@ -9978,7 +10083,7 @@
         <v>46215</v>
       </c>
     </row>
-    <row r="449" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A449" s="5" t="s">
         <v>146</v>
       </c>
@@ -9998,7 +10103,7 @@
         <v>46215</v>
       </c>
     </row>
-    <row r="450" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A450" s="4" t="s">
         <v>28</v>
       </c>
@@ -10018,7 +10123,7 @@
         <v>46215</v>
       </c>
     </row>
-    <row r="451" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A451" s="4" t="s">
         <v>28</v>
       </c>
@@ -10031,14 +10136,14 @@
       <c r="D451" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E451" s="12" t="s">
+      <c r="E451" s="4" t="s">
         <v>164</v>
       </c>
       <c r="F451" s="9">
         <v>46215</v>
       </c>
     </row>
-    <row r="452" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A452" s="4" t="s">
         <v>28</v>
       </c>
@@ -10051,14 +10156,14 @@
       <c r="D452" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="E452" s="12" t="s">
+      <c r="E452" s="4" t="s">
         <v>164</v>
       </c>
       <c r="F452" s="9">
         <v>46215</v>
       </c>
     </row>
-    <row r="453" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A453" s="5" t="s">
         <v>116</v>
       </c>
@@ -10079,7 +10184,7 @@
       </c>
       <c r="G453" s="10"/>
     </row>
-    <row r="454" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A454" s="5" t="s">
         <v>116</v>
       </c>
@@ -10100,7 +10205,7 @@
       </c>
       <c r="G454" s="10"/>
     </row>
-    <row r="455" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A455" s="4" t="s">
         <v>146</v>
       </c>
@@ -10113,14 +10218,14 @@
       <c r="D455" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E455" s="12" t="s">
+      <c r="E455" s="4" t="s">
         <v>164</v>
       </c>
       <c r="F455" s="9">
         <v>46216</v>
       </c>
     </row>
-    <row r="456" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A456" s="4" t="s">
         <v>146</v>
       </c>
@@ -10133,14 +10238,14 @@
       <c r="D456" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E456" s="12" t="s">
+      <c r="E456" s="4" t="s">
         <v>164</v>
       </c>
       <c r="F456" s="9">
         <v>46216</v>
       </c>
     </row>
-    <row r="457" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A457" s="5" t="s">
         <v>116</v>
       </c>
@@ -10160,7 +10265,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="458" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A458" s="5" t="s">
         <v>116</v>
       </c>
@@ -10180,7 +10285,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="459" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A459" s="5" t="s">
         <v>116</v>
       </c>
@@ -10200,7 +10305,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="460" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A460" s="4" t="s">
         <v>166</v>
       </c>
@@ -10213,14 +10318,14 @@
       <c r="D460" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E460" s="12" t="s">
+      <c r="E460" s="4" t="s">
         <v>164</v>
       </c>
       <c r="F460" s="9">
         <v>46218</v>
       </c>
     </row>
-    <row r="461" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A461" s="4" t="s">
         <v>166</v>
       </c>
@@ -10233,14 +10338,14 @@
       <c r="D461" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E461" s="12" t="s">
+      <c r="E461" s="4" t="s">
         <v>164</v>
       </c>
       <c r="F461" s="9">
         <v>46218</v>
       </c>
     </row>
-    <row r="462" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A462" s="4" t="s">
         <v>166</v>
       </c>
@@ -10253,20 +10358,854 @@
       <c r="D462" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E462" s="12" t="s">
+      <c r="E462" s="4" t="s">
         <v>164</v>
       </c>
       <c r="F462" s="9">
         <v>46218</v>
       </c>
-    </row>
-    <row r="463" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A463" s="11"/>
-      <c r="B463" s="11"/>
-      <c r="C463" s="11"/>
-      <c r="D463" s="11"/>
-      <c r="E463" s="13"/>
-      <c r="F463" s="11"/>
+      <c r="G462" s="10"/>
+      <c r="H462" s="10"/>
+    </row>
+    <row r="463" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A463" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="B463" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="C463" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D463" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E463" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="F463" s="13">
+        <v>46219</v>
+      </c>
+      <c r="G463" s="10"/>
+      <c r="H463" s="10"/>
+    </row>
+    <row r="464" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A464" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="B464" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="C464" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D464" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E464" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="F464" s="13">
+        <v>46219</v>
+      </c>
+      <c r="G464" s="10"/>
+      <c r="H464" s="10"/>
+    </row>
+    <row r="465" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A465" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="B465" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="C465" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D465" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E465" s="11"/>
+      <c r="F465" s="11"/>
+      <c r="G465" s="10"/>
+      <c r="H465" s="10"/>
+    </row>
+    <row r="466" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A466" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="B466" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="C466" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D466" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E466" s="11"/>
+      <c r="F466" s="11"/>
+      <c r="G466" s="10"/>
+      <c r="H466" s="10"/>
+    </row>
+    <row r="467" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A467" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="B467" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="C467" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="D467" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="E467" s="11"/>
+      <c r="F467" s="11"/>
+      <c r="G467" s="10"/>
+      <c r="H467" s="10"/>
+    </row>
+    <row r="468" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A468" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="B468" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="C468" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D468" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E468" s="11"/>
+      <c r="F468" s="11"/>
+      <c r="G468" s="10"/>
+      <c r="H468" s="10"/>
+    </row>
+    <row r="469" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A469" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="B469" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="C469" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="D469" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E469" s="11"/>
+      <c r="F469" s="11"/>
+      <c r="G469" s="10"/>
+      <c r="H469" s="10"/>
+    </row>
+    <row r="470" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A470" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="B470" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="C470" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D470" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E470" s="11"/>
+      <c r="F470" s="11"/>
+    </row>
+    <row r="471" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A471" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B471" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="C471" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D471" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E471" s="11"/>
+      <c r="F471" s="11"/>
+    </row>
+    <row r="472" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A472" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B472" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="C472" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D472" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E472" s="11"/>
+      <c r="F472" s="11"/>
+    </row>
+    <row r="473" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A473" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B473" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="C473" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D473" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E473" s="11"/>
+      <c r="F473" s="11"/>
+    </row>
+    <row r="474" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A474" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B474" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="C474" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="D474" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="E474" s="11"/>
+      <c r="F474" s="11"/>
+    </row>
+    <row r="475" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A475" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B475" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C475" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D475" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E475" s="11"/>
+      <c r="F475" s="11"/>
+    </row>
+    <row r="476" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A476" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B476" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C476" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D476" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E476" s="11"/>
+      <c r="F476" s="11"/>
+    </row>
+    <row r="477" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A477" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B477" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C477" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D477" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E477" s="11"/>
+      <c r="F477" s="11"/>
+    </row>
+    <row r="478" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A478" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="B478" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="C478" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D478" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E478" s="11"/>
+      <c r="F478" s="11"/>
+      <c r="G478" s="12"/>
+    </row>
+    <row r="479" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A479" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="B479" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="C479" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D479" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E479" s="11"/>
+      <c r="F479" s="11"/>
+      <c r="G479" s="12"/>
+    </row>
+    <row r="480" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A480" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="B480" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="C480" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D480" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E480" s="11"/>
+      <c r="F480" s="11"/>
+      <c r="G480" s="12"/>
+    </row>
+    <row r="481" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A481" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="B481" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="C481" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="D481" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E481" s="11"/>
+      <c r="F481" s="11"/>
+      <c r="G481" s="12"/>
+    </row>
+    <row r="482" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A482" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="B482" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="C482" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D482" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E482" s="11"/>
+      <c r="F482" s="11"/>
+      <c r="G482" s="12"/>
+    </row>
+    <row r="483" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A483" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="B483" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="C483" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="D483" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="E483" s="11"/>
+      <c r="F483" s="11"/>
+      <c r="G483" s="12"/>
+    </row>
+    <row r="484" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A484" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="B484" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="C484" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D484" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="E484" s="11"/>
+      <c r="F484" s="11"/>
+      <c r="G484" s="12"/>
+    </row>
+    <row r="485" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A485" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="B485" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="C485" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D485" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E485" s="11"/>
+      <c r="F485" s="11"/>
+      <c r="G485" s="12"/>
+    </row>
+    <row r="486" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A486" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="B486" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="C486" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="D486" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E486" s="11"/>
+      <c r="F486" s="11"/>
+      <c r="G486" s="12"/>
+    </row>
+    <row r="487" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A487" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="B487" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="C487" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D487" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E487" s="11"/>
+      <c r="F487" s="11"/>
+      <c r="G487" s="12"/>
+    </row>
+    <row r="488" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A488" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="B488" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="C488" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D488" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E488" s="11"/>
+      <c r="F488" s="11"/>
+      <c r="G488" s="12"/>
+    </row>
+    <row r="489" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A489" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="B489" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C489" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="D489" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E489" s="11"/>
+      <c r="F489" s="11"/>
+      <c r="G489" s="12"/>
+    </row>
+    <row r="490" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A490" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="B490" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C490" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D490" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="E490" s="11"/>
+      <c r="F490" s="11"/>
+      <c r="G490" s="12"/>
+    </row>
+    <row r="491" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A491" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="B491" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C491" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="D491" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E491" s="11"/>
+      <c r="F491" s="11"/>
+      <c r="G491" s="12"/>
+    </row>
+    <row r="492" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A492" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="B492" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="C492" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D492" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E492" s="11"/>
+      <c r="F492" s="11"/>
+      <c r="G492" s="12"/>
+    </row>
+    <row r="493" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A493" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="B493" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="C493" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D493" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E493" s="11"/>
+      <c r="F493" s="11"/>
+      <c r="G493" s="12"/>
+    </row>
+    <row r="494" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A494" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B494" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="C494" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D494" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E494" s="11"/>
+      <c r="F494" s="11"/>
+      <c r="G494" s="12"/>
+    </row>
+    <row r="495" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A495" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B495" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="C495" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D495" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E495" s="11"/>
+      <c r="F495" s="11"/>
+      <c r="G495" s="12"/>
+    </row>
+    <row r="496" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A496" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B496" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="C496" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="D496" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="E496" s="11"/>
+      <c r="F496" s="11"/>
+      <c r="G496" s="12"/>
+    </row>
+    <row r="497" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A497" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="B497" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="C497" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D497" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E497" s="11"/>
+      <c r="F497" s="11"/>
+      <c r="G497" s="12"/>
+    </row>
+    <row r="498" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A498" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="B498" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="C498" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D498" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E498" s="11"/>
+      <c r="F498" s="11"/>
+      <c r="G498" s="12"/>
+    </row>
+    <row r="499" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A499" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="B499" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="C499" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D499" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E499" s="11"/>
+      <c r="F499" s="11"/>
+      <c r="G499" s="12"/>
+    </row>
+    <row r="500" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A500" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="B500" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="C500" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D500" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E500" s="11"/>
+      <c r="F500" s="11"/>
+      <c r="G500" s="12"/>
+    </row>
+    <row r="501" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A501" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B501" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="C501" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D501" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E501" s="11"/>
+      <c r="F501" s="11"/>
+      <c r="G501" s="12"/>
+    </row>
+    <row r="502" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A502" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B502" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="C502" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D502" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E502" s="11"/>
+      <c r="F502" s="11"/>
+      <c r="G502" s="12"/>
+    </row>
+    <row r="503" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A503" s="11"/>
+      <c r="B503" s="11"/>
+      <c r="C503" s="11"/>
+      <c r="D503" s="11"/>
+      <c r="E503" s="11"/>
+      <c r="F503" s="11"/>
+      <c r="G503" s="12"/>
+    </row>
+    <row r="504" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A504" s="11"/>
+      <c r="B504" s="11"/>
+      <c r="C504" s="11"/>
+      <c r="D504" s="11"/>
+      <c r="E504" s="11"/>
+      <c r="F504" s="11"/>
+      <c r="G504" s="12"/>
+    </row>
+    <row r="505" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A505" s="11"/>
+      <c r="B505" s="11"/>
+      <c r="C505" s="11"/>
+      <c r="D505" s="11"/>
+      <c r="E505" s="11"/>
+      <c r="F505" s="11"/>
+      <c r="G505" s="12"/>
+    </row>
+    <row r="506" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A506" s="11"/>
+      <c r="B506" s="11"/>
+      <c r="C506" s="11"/>
+      <c r="D506" s="11"/>
+      <c r="E506" s="11"/>
+      <c r="F506" s="11"/>
+      <c r="G506" s="12"/>
+    </row>
+    <row r="507" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A507" s="11"/>
+      <c r="B507" s="11"/>
+      <c r="C507" s="11"/>
+      <c r="D507" s="11"/>
+      <c r="E507" s="11"/>
+      <c r="F507" s="11"/>
+      <c r="G507" s="12"/>
+    </row>
+    <row r="508" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A508" s="11"/>
+      <c r="B508" s="11"/>
+      <c r="C508" s="11"/>
+      <c r="D508" s="11"/>
+      <c r="E508" s="11"/>
+      <c r="F508" s="11"/>
+      <c r="G508" s="12"/>
+    </row>
+    <row r="509" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A509" s="11"/>
+      <c r="B509" s="11"/>
+      <c r="C509" s="11"/>
+      <c r="D509" s="11"/>
+      <c r="E509" s="11"/>
+      <c r="F509" s="11"/>
+      <c r="G509" s="12"/>
+    </row>
+    <row r="510" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A510" s="11"/>
+      <c r="B510" s="11"/>
+      <c r="C510" s="11"/>
+      <c r="D510" s="11"/>
+      <c r="E510" s="11"/>
+      <c r="F510" s="11"/>
+      <c r="G510" s="12"/>
+    </row>
+    <row r="511" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A511" s="11"/>
+      <c r="B511" s="11"/>
+      <c r="C511" s="11"/>
+      <c r="D511" s="11"/>
+      <c r="E511" s="11"/>
+      <c r="F511" s="11"/>
+      <c r="G511" s="12"/>
+    </row>
+    <row r="512" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A512" s="11"/>
+      <c r="B512" s="11"/>
+      <c r="C512" s="11"/>
+      <c r="D512" s="11"/>
+      <c r="E512" s="11"/>
+      <c r="F512" s="11"/>
+      <c r="G512" s="12"/>
+    </row>
+    <row r="513" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A513" s="11"/>
+      <c r="B513" s="11"/>
+      <c r="C513" s="11"/>
+      <c r="D513" s="11"/>
+      <c r="E513" s="11"/>
+      <c r="F513" s="11"/>
+      <c r="G513" s="12"/>
+    </row>
+    <row r="514" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A514" s="11"/>
+      <c r="B514" s="11"/>
+      <c r="C514" s="11"/>
+      <c r="D514" s="11"/>
+      <c r="E514" s="11"/>
+      <c r="F514" s="11"/>
+      <c r="G514" s="12"/>
+    </row>
+    <row r="515" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A515" s="11"/>
+      <c r="B515" s="11"/>
+      <c r="C515" s="11"/>
+      <c r="D515" s="11"/>
+      <c r="E515" s="11"/>
+      <c r="F515" s="11"/>
+      <c r="G515" s="12"/>
+    </row>
+    <row r="516" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A516" s="11"/>
+      <c r="B516" s="11"/>
+      <c r="C516" s="11"/>
+      <c r="D516" s="11"/>
+      <c r="E516" s="11"/>
+      <c r="F516" s="11"/>
+      <c r="G516" s="12"/>
+    </row>
+    <row r="517" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A517" s="11"/>
+      <c r="B517" s="11"/>
+      <c r="C517" s="11"/>
+      <c r="D517" s="11"/>
+      <c r="E517" s="11"/>
+      <c r="F517" s="11"/>
+      <c r="G517" s="12"/>
+    </row>
+    <row r="518" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A518" s="11"/>
+      <c r="B518" s="11"/>
+      <c r="C518" s="11"/>
+      <c r="D518" s="11"/>
+      <c r="E518" s="11"/>
+      <c r="F518" s="11"/>
+      <c r="G518" s="12"/>
+    </row>
+    <row r="519" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A519" s="11"/>
+      <c r="B519" s="11"/>
+      <c r="C519" s="11"/>
+      <c r="D519" s="11"/>
+      <c r="E519" s="11"/>
+      <c r="F519" s="11"/>
+      <c r="G519" s="12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Winamax Spanish Circuit 2 - Stage 2
</commit_message>
<xml_diff>
--- a/file/history.xlsx
+++ b/file/history.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/faa3f9bfbb5dc780/Documentos/GitHub/ck-tools/file/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="13_ncr:1_{AB7ADBC0-0AFC-4EB5-BDC6-F57936754D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAE06C51-1287-4C3D-8F99-72B017C589A6}"/>
+  <xr:revisionPtr revIDLastSave="310" documentId="13_ncr:1_{AB7ADBC0-0AFC-4EB5-BDC6-F57936754D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EA92924-92A5-49A4-93CE-EF44D84367BC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{39BF18F1-6CA4-42F4-B020-2D59954264FB}"/>
+    <workbookView xWindow="3195" yWindow="1785" windowWidth="23250" windowHeight="12450" xr2:uid="{39BF18F1-6CA4-42F4-B020-2D59954264FB}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2473" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2601" uniqueCount="266">
   <si>
     <t>Team 1</t>
   </si>
@@ -663,6 +663,177 @@
   </si>
   <si>
     <t>Vox Eminor</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2027</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2028</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2029</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2030</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2031</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2032</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2033</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2034</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2035</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2036</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2037</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2038</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2039</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2040</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2041</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2042</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2043</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2044</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2045</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2046</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2047</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2048</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2049</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2050</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2051</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2052</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2053</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2054</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2055</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2056</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2057</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2058</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2059</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2060</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2061</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2062</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2063</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2064</t>
+  </si>
+  <si>
+    <t>13x</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2065</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2066</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2067</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2068</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2069</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2070</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2071</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2072</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2073</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2074</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2075</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2076</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2077</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2078</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2079</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2080</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2081</t>
+  </si>
+  <si>
+    <t>Winamax Spanish Cirtuit 2082</t>
   </si>
 </sst>
 </file>
@@ -737,7 +908,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -771,9 +942,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -789,6 +957,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1108,7 +1280,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECD49EDF-97AD-42E2-9203-75390A90C7F2}">
-  <dimension ref="A1:H519"/>
+  <dimension ref="A1:H533"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" style="1" customWidth="1"/>
@@ -10368,844 +10540,1324 @@
       <c r="H462" s="10"/>
     </row>
     <row r="463" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A463" s="11" t="s">
+      <c r="A463" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="B463" s="11" t="s">
+      <c r="B463" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C463" s="11" t="s">
+      <c r="C463" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D463" s="11" t="s">
+      <c r="D463" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E463" s="11" t="s">
+      <c r="E463" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="F463" s="13">
+      <c r="F463" s="8">
         <v>46219</v>
       </c>
       <c r="G463" s="10"/>
       <c r="H463" s="10"/>
     </row>
     <row r="464" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A464" s="11" t="s">
+      <c r="A464" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="B464" s="11" t="s">
+      <c r="B464" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C464" s="11" t="s">
+      <c r="C464" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D464" s="11" t="s">
+      <c r="D464" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E464" s="11" t="s">
+      <c r="E464" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="F464" s="13">
+      <c r="F464" s="8">
         <v>46219</v>
       </c>
       <c r="G464" s="10"/>
       <c r="H464" s="10"/>
     </row>
     <row r="465" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A465" s="11" t="s">
+      <c r="A465" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B465" s="11" t="s">
+      <c r="B465" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C465" s="11" t="s">
+      <c r="C465" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D465" s="11" t="s">
+      <c r="D465" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E465" s="11"/>
-      <c r="F465" s="11"/>
+      <c r="E465" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="F465" s="9">
+        <v>46219</v>
+      </c>
       <c r="G465" s="10"/>
       <c r="H465" s="10"/>
     </row>
     <row r="466" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A466" s="11" t="s">
+      <c r="A466" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B466" s="11" t="s">
+      <c r="B466" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C466" s="11" t="s">
+      <c r="C466" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D466" s="11" t="s">
+      <c r="D466" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E466" s="11"/>
-      <c r="F466" s="11"/>
+      <c r="E466" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="F466" s="9">
+        <v>46219</v>
+      </c>
       <c r="G466" s="10"/>
       <c r="H466" s="10"/>
     </row>
     <row r="467" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A467" s="11" t="s">
+      <c r="A467" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B467" s="11" t="s">
+      <c r="B467" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C467" s="11" t="s">
+      <c r="C467" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D467" s="11" t="s">
+      <c r="D467" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="E467" s="11"/>
-      <c r="F467" s="11"/>
+      <c r="E467" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="F467" s="9">
+        <v>46219</v>
+      </c>
       <c r="G467" s="10"/>
       <c r="H467" s="10"/>
     </row>
     <row r="468" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A468" s="11" t="s">
+      <c r="A468" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="B468" s="11" t="s">
+      <c r="B468" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="C468" s="11" t="s">
+      <c r="C468" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D468" s="11" t="s">
+      <c r="D468" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E468" s="11"/>
-      <c r="F468" s="11"/>
+      <c r="E468" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="F468" s="8">
+        <v>46219</v>
+      </c>
       <c r="G468" s="10"/>
       <c r="H468" s="10"/>
     </row>
     <row r="469" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A469" s="11" t="s">
+      <c r="A469" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="B469" s="11" t="s">
+      <c r="B469" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="C469" s="11" t="s">
+      <c r="C469" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D469" s="11" t="s">
+      <c r="D469" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E469" s="11"/>
-      <c r="F469" s="11"/>
+      <c r="E469" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="F469" s="8">
+        <v>46219</v>
+      </c>
       <c r="G469" s="10"/>
       <c r="H469" s="10"/>
     </row>
     <row r="470" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A470" s="11" t="s">
+      <c r="A470" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="B470" s="11" t="s">
+      <c r="B470" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="C470" s="11" t="s">
+      <c r="C470" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D470" s="11" t="s">
+      <c r="D470" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E470" s="11"/>
-      <c r="F470" s="11"/>
+      <c r="E470" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F470" s="8">
+        <v>46219</v>
+      </c>
     </row>
     <row r="471" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A471" s="11" t="s">
+      <c r="A471" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="B471" s="11" t="s">
+      <c r="B471" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="C471" s="11" t="s">
+      <c r="C471" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D471" s="11" t="s">
+      <c r="D471" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E471" s="11"/>
-      <c r="F471" s="11"/>
+      <c r="E471" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="F471" s="9">
+        <v>46219</v>
+      </c>
     </row>
     <row r="472" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A472" s="11" t="s">
+      <c r="A472" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="B472" s="11" t="s">
+      <c r="B472" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="C472" s="11" t="s">
+      <c r="C472" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D472" s="11" t="s">
+      <c r="D472" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E472" s="11"/>
-      <c r="F472" s="11"/>
+      <c r="E472" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="F472" s="9">
+        <v>46219</v>
+      </c>
     </row>
     <row r="473" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A473" s="11" t="s">
+      <c r="A473" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="B473" s="11" t="s">
+      <c r="B473" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="C473" s="11" t="s">
+      <c r="C473" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D473" s="11" t="s">
+      <c r="D473" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E473" s="11"/>
-      <c r="F473" s="11"/>
+      <c r="E473" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="F473" s="8">
+        <v>46219</v>
+      </c>
     </row>
     <row r="474" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A474" s="11" t="s">
+      <c r="A474" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="B474" s="11" t="s">
+      <c r="B474" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="C474" s="11" t="s">
+      <c r="C474" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="D474" s="11" t="s">
+      <c r="D474" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="E474" s="11"/>
-      <c r="F474" s="11"/>
+      <c r="E474" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="F474" s="8">
+        <v>46219</v>
+      </c>
     </row>
     <row r="475" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A475" s="11" t="s">
+      <c r="A475" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="B475" s="11" t="s">
+      <c r="B475" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="C475" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D475" s="11" t="s">
+      <c r="C475" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D475" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E475" s="11"/>
-      <c r="F475" s="11"/>
+      <c r="E475" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="F475" s="9">
+        <v>46219</v>
+      </c>
     </row>
     <row r="476" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A476" s="11" t="s">
+      <c r="A476" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="B476" s="11" t="s">
+      <c r="B476" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="C476" s="11" t="s">
+      <c r="C476" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D476" s="11" t="s">
+      <c r="D476" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E476" s="11"/>
-      <c r="F476" s="11"/>
+      <c r="E476" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="F476" s="9">
+        <v>46219</v>
+      </c>
     </row>
     <row r="477" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A477" s="11" t="s">
+      <c r="A477" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="B477" s="11" t="s">
+      <c r="B477" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="C477" s="11" t="s">
+      <c r="C477" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D477" s="11" t="s">
+      <c r="D477" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="E477" s="11"/>
-      <c r="F477" s="11"/>
+      <c r="E477" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="F477" s="9">
+        <v>46219</v>
+      </c>
     </row>
     <row r="478" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A478" s="11" t="s">
+      <c r="A478" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="B478" s="11" t="s">
+      <c r="B478" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C478" s="11" t="s">
+      <c r="C478" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D478" s="11" t="s">
+      <c r="D478" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E478" s="11"/>
-      <c r="F478" s="11"/>
+      <c r="E478" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="F478" s="8">
+        <v>46220</v>
+      </c>
       <c r="G478" s="12"/>
     </row>
     <row r="479" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A479" s="11" t="s">
+      <c r="A479" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="B479" s="11" t="s">
+      <c r="B479" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C479" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D479" s="11" t="s">
+      <c r="C479" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D479" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="E479" s="11"/>
-      <c r="F479" s="11"/>
+      <c r="E479" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="F479" s="8">
+        <v>46220</v>
+      </c>
       <c r="G479" s="12"/>
     </row>
     <row r="480" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A480" s="11" t="s">
+      <c r="A480" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B480" s="11" t="s">
+      <c r="B480" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C480" s="11" t="s">
+      <c r="C480" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D480" s="11" t="s">
+      <c r="D480" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E480" s="11"/>
-      <c r="F480" s="11"/>
+      <c r="E480" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="F480" s="9">
+        <v>46220</v>
+      </c>
       <c r="G480" s="12"/>
     </row>
     <row r="481" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A481" s="11" t="s">
+      <c r="A481" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B481" s="11" t="s">
+      <c r="B481" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C481" s="11" t="s">
+      <c r="C481" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D481" s="11" t="s">
+      <c r="D481" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E481" s="11"/>
-      <c r="F481" s="11"/>
+      <c r="E481" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="F481" s="9">
+        <v>46220</v>
+      </c>
       <c r="G481" s="12"/>
     </row>
     <row r="482" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A482" s="11" t="s">
+      <c r="A482" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B482" s="11" t="s">
+      <c r="B482" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C482" s="11" t="s">
+      <c r="C482" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D482" s="11" t="s">
+      <c r="D482" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E482" s="11"/>
-      <c r="F482" s="11"/>
+      <c r="E482" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="F482" s="9">
+        <v>46220</v>
+      </c>
       <c r="G482" s="12"/>
     </row>
     <row r="483" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A483" s="11" t="s">
+      <c r="A483" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="B483" s="11" t="s">
+      <c r="B483" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="C483" s="11" t="s">
+      <c r="C483" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D483" s="11" t="s">
+      <c r="D483" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="E483" s="11"/>
-      <c r="F483" s="11"/>
+      <c r="E483" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="F483" s="8">
+        <v>46220</v>
+      </c>
       <c r="G483" s="12"/>
     </row>
     <row r="484" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A484" s="11" t="s">
+      <c r="A484" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="B484" s="11" t="s">
+      <c r="B484" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="C484" s="11" t="s">
+      <c r="C484" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D484" s="11" t="s">
+      <c r="D484" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="E484" s="11"/>
-      <c r="F484" s="11"/>
+      <c r="E484" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="F484" s="8">
+        <v>46220</v>
+      </c>
       <c r="G484" s="12"/>
     </row>
     <row r="485" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A485" s="11" t="s">
+      <c r="A485" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="B485" s="11" t="s">
+      <c r="B485" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="C485" s="11" t="s">
+      <c r="C485" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D485" s="11" t="s">
+      <c r="D485" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E485" s="11"/>
-      <c r="F485" s="11"/>
+      <c r="E485" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="F485" s="8">
+        <v>46220</v>
+      </c>
       <c r="G485" s="12"/>
     </row>
     <row r="486" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A486" s="11" t="s">
+      <c r="A486" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="B486" s="11" t="s">
+      <c r="B486" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="C486" s="11" t="s">
+      <c r="C486" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D486" s="11" t="s">
+      <c r="D486" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E486" s="11"/>
-      <c r="F486" s="11"/>
+      <c r="E486" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="F486" s="9">
+        <v>46220</v>
+      </c>
       <c r="G486" s="12"/>
     </row>
     <row r="487" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A487" s="11" t="s">
+      <c r="A487" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="B487" s="11" t="s">
+      <c r="B487" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="C487" s="11" t="s">
+      <c r="C487" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D487" s="11" t="s">
+      <c r="D487" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E487" s="11"/>
-      <c r="F487" s="11"/>
+      <c r="E487" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="F487" s="9">
+        <v>46220</v>
+      </c>
       <c r="G487" s="12"/>
     </row>
     <row r="488" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A488" s="11" t="s">
+      <c r="A488" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="B488" s="11" t="s">
+      <c r="B488" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="C488" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D488" s="11" t="s">
+      <c r="C488" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D488" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E488" s="11"/>
-      <c r="F488" s="11"/>
+      <c r="E488" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="F488" s="9">
+        <v>46220</v>
+      </c>
       <c r="G488" s="12"/>
     </row>
     <row r="489" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A489" s="11" t="s">
+      <c r="A489" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="B489" s="11" t="s">
+      <c r="B489" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="C489" s="11" t="s">
+      <c r="C489" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D489" s="11" t="s">
+      <c r="D489" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E489" s="11"/>
-      <c r="F489" s="11"/>
+      <c r="E489" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="F489" s="8">
+        <v>46220</v>
+      </c>
       <c r="G489" s="12"/>
     </row>
     <row r="490" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A490" s="11" t="s">
+      <c r="A490" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="B490" s="11" t="s">
+      <c r="B490" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="C490" s="11" t="s">
+      <c r="C490" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D490" s="11" t="s">
+      <c r="D490" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="E490" s="11"/>
-      <c r="F490" s="11"/>
+      <c r="E490" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="F490" s="8">
+        <v>46220</v>
+      </c>
       <c r="G490" s="12"/>
     </row>
     <row r="491" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A491" s="11" t="s">
+      <c r="A491" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="B491" s="11" t="s">
+      <c r="B491" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="C491" s="11" t="s">
+      <c r="C491" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="D491" s="11" t="s">
+      <c r="D491" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E491" s="11"/>
-      <c r="F491" s="11"/>
+      <c r="E491" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="F491" s="8">
+        <v>46220</v>
+      </c>
       <c r="G491" s="12"/>
     </row>
     <row r="492" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A492" s="11" t="s">
+      <c r="A492" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="B492" s="11" t="s">
+      <c r="B492" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C492" s="11" t="s">
+      <c r="C492" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D492" s="11" t="s">
+      <c r="D492" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E492" s="11"/>
-      <c r="F492" s="11"/>
+      <c r="E492" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F492" s="9">
+        <v>46220</v>
+      </c>
       <c r="G492" s="12"/>
     </row>
     <row r="493" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A493" s="11" t="s">
+      <c r="A493" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="B493" s="11" t="s">
+      <c r="B493" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C493" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D493" s="11" t="s">
+      <c r="C493" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D493" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E493" s="11"/>
-      <c r="F493" s="11"/>
+      <c r="E493" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="F493" s="9">
+        <v>46220</v>
+      </c>
       <c r="G493" s="12"/>
     </row>
     <row r="494" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A494" s="11" t="s">
+      <c r="A494" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="B494" s="11" t="s">
+      <c r="B494" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="C494" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D494" s="11" t="s">
+      <c r="C494" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D494" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E494" s="11"/>
-      <c r="F494" s="11"/>
+      <c r="E494" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="F494" s="8">
+        <v>46220</v>
+      </c>
       <c r="G494" s="12"/>
     </row>
     <row r="495" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A495" s="11" t="s">
+      <c r="A495" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="B495" s="11" t="s">
+      <c r="B495" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="C495" s="11" t="s">
+      <c r="C495" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D495" s="11" t="s">
+      <c r="D495" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E495" s="11"/>
-      <c r="F495" s="11"/>
+      <c r="E495" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="F495" s="8">
+        <v>46220</v>
+      </c>
       <c r="G495" s="12"/>
     </row>
     <row r="496" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A496" s="11" t="s">
+      <c r="A496" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="B496" s="11" t="s">
+      <c r="B496" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="C496" s="11" t="s">
+      <c r="C496" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="D496" s="11" t="s">
+      <c r="D496" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="E496" s="11"/>
-      <c r="F496" s="11"/>
+      <c r="E496" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="F496" s="8">
+        <v>46220</v>
+      </c>
       <c r="G496" s="12"/>
     </row>
     <row r="497" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A497" s="11" t="s">
+      <c r="A497" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="B497" s="11" t="s">
+      <c r="B497" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="C497" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D497" s="11" t="s">
+      <c r="C497" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D497" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E497" s="11"/>
-      <c r="F497" s="11"/>
+      <c r="E497" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="F497" s="9">
+        <v>46221</v>
+      </c>
       <c r="G497" s="12"/>
     </row>
     <row r="498" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A498" s="11" t="s">
+      <c r="A498" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="B498" s="11" t="s">
+      <c r="B498" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="C498" s="11" t="s">
+      <c r="C498" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D498" s="11" t="s">
+      <c r="D498" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E498" s="11"/>
-      <c r="F498" s="11"/>
+      <c r="E498" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="F498" s="9">
+        <v>46221</v>
+      </c>
       <c r="G498" s="12"/>
     </row>
     <row r="499" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A499" s="11" t="s">
+      <c r="A499" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="B499" s="11" t="s">
+      <c r="B499" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="C499" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D499" s="11" t="s">
+      <c r="C499" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D499" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="E499" s="11"/>
-      <c r="F499" s="11"/>
+      <c r="E499" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="F499" s="8">
+        <v>46221</v>
+      </c>
       <c r="G499" s="12"/>
     </row>
     <row r="500" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A500" s="11" t="s">
+      <c r="A500" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="B500" s="11" t="s">
+      <c r="B500" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="C500" s="11" t="s">
+      <c r="C500" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D500" s="11" t="s">
+      <c r="D500" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E500" s="11"/>
-      <c r="F500" s="11"/>
+      <c r="E500" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="F500" s="8">
+        <v>46221</v>
+      </c>
       <c r="G500" s="12"/>
     </row>
     <row r="501" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A501" s="11" t="s">
+      <c r="A501" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="B501" s="11" t="s">
+      <c r="B501" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="C501" s="11" t="s">
+      <c r="C501" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D501" s="11" t="s">
+      <c r="D501" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E501" s="11"/>
-      <c r="F501" s="11"/>
+      <c r="E501" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="F501" s="9">
+        <v>46221</v>
+      </c>
       <c r="G501" s="12"/>
     </row>
     <row r="502" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A502" s="11" t="s">
+      <c r="A502" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="B502" s="11" t="s">
+      <c r="B502" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="C502" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D502" s="11" t="s">
+      <c r="C502" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D502" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E502" s="11"/>
-      <c r="F502" s="11"/>
+      <c r="E502" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F502" s="9">
+        <v>46221</v>
+      </c>
       <c r="G502" s="12"/>
     </row>
     <row r="503" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A503" s="11"/>
-      <c r="B503" s="11"/>
-      <c r="C503" s="11"/>
-      <c r="D503" s="11"/>
-      <c r="E503" s="11"/>
-      <c r="F503" s="11"/>
+      <c r="A503" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B503" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="C503" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D503" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="E503" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F503" s="9">
+        <v>46225</v>
+      </c>
       <c r="G503" s="12"/>
     </row>
     <row r="504" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A504" s="11"/>
-      <c r="B504" s="11"/>
-      <c r="C504" s="11"/>
-      <c r="D504" s="11"/>
-      <c r="E504" s="11"/>
-      <c r="F504" s="11"/>
+      <c r="A504" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B504" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="C504" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D504" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E504" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="F504" s="9">
+        <v>46225</v>
+      </c>
       <c r="G504" s="12"/>
     </row>
     <row r="505" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A505" s="11"/>
-      <c r="B505" s="11"/>
-      <c r="C505" s="11"/>
-      <c r="D505" s="11"/>
-      <c r="E505" s="11"/>
-      <c r="F505" s="11"/>
+      <c r="A505" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B505" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C505" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D505" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E505" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="F505" s="9">
+        <v>46225</v>
+      </c>
       <c r="G505" s="12"/>
     </row>
     <row r="506" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A506" s="11"/>
-      <c r="B506" s="11"/>
-      <c r="C506" s="11"/>
-      <c r="D506" s="11"/>
-      <c r="E506" s="11"/>
-      <c r="F506" s="11"/>
+      <c r="A506" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B506" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C506" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D506" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E506" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="F506" s="9">
+        <v>46225</v>
+      </c>
       <c r="G506" s="12"/>
     </row>
     <row r="507" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A507" s="11"/>
-      <c r="B507" s="11"/>
-      <c r="C507" s="11"/>
-      <c r="D507" s="11"/>
-      <c r="E507" s="11"/>
-      <c r="F507" s="11"/>
+      <c r="A507" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B507" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C507" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D507" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E507" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F507" s="9">
+        <v>46225</v>
+      </c>
       <c r="G507" s="12"/>
     </row>
     <row r="508" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A508" s="11"/>
-      <c r="B508" s="11"/>
-      <c r="C508" s="11"/>
-      <c r="D508" s="11"/>
-      <c r="E508" s="11"/>
-      <c r="F508" s="11"/>
+      <c r="A508" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B508" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="C508" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D508" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E508" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="F508" s="9">
+        <v>46226</v>
+      </c>
       <c r="G508" s="12"/>
     </row>
     <row r="509" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A509" s="11"/>
-      <c r="B509" s="11"/>
-      <c r="C509" s="11"/>
-      <c r="D509" s="11"/>
-      <c r="E509" s="11"/>
-      <c r="F509" s="11"/>
+      <c r="A509" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B509" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="C509" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D509" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E509" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="F509" s="9">
+        <v>46226</v>
+      </c>
       <c r="G509" s="12"/>
     </row>
     <row r="510" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A510" s="11"/>
-      <c r="B510" s="11"/>
-      <c r="C510" s="11"/>
-      <c r="D510" s="11"/>
-      <c r="E510" s="11"/>
-      <c r="F510" s="11"/>
+      <c r="A510" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B510" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C510" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D510" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E510" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="F510" s="9">
+        <v>46226</v>
+      </c>
       <c r="G510" s="12"/>
     </row>
     <row r="511" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A511" s="11"/>
-      <c r="B511" s="11"/>
-      <c r="C511" s="11"/>
-      <c r="D511" s="11"/>
-      <c r="E511" s="11"/>
-      <c r="F511" s="11"/>
+      <c r="A511" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B511" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C511" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D511" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E511" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F511" s="9">
+        <v>46226</v>
+      </c>
       <c r="G511" s="12"/>
     </row>
     <row r="512" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A512" s="11"/>
-      <c r="B512" s="11"/>
-      <c r="C512" s="11"/>
-      <c r="D512" s="11"/>
-      <c r="E512" s="11"/>
-      <c r="F512" s="11"/>
+      <c r="A512" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B512" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C512" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D512" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E512" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="F512" s="9">
+        <v>46226</v>
+      </c>
       <c r="G512" s="12"/>
     </row>
     <row r="513" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A513" s="11"/>
-      <c r="B513" s="11"/>
-      <c r="C513" s="11"/>
-      <c r="D513" s="11"/>
-      <c r="E513" s="11"/>
-      <c r="F513" s="11"/>
+      <c r="A513" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B513" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C513" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D513" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E513" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="F513" s="9">
+        <v>46226</v>
+      </c>
       <c r="G513" s="12"/>
     </row>
     <row r="514" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A514" s="11"/>
-      <c r="B514" s="11"/>
-      <c r="C514" s="11"/>
-      <c r="D514" s="11"/>
-      <c r="E514" s="11"/>
-      <c r="F514" s="11"/>
+      <c r="A514" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B514" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C514" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D514" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="E514" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="F514" s="9">
+        <v>46226</v>
+      </c>
       <c r="G514" s="12"/>
     </row>
     <row r="515" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A515" s="11"/>
-      <c r="B515" s="11"/>
-      <c r="C515" s="11"/>
-      <c r="D515" s="11"/>
-      <c r="E515" s="11"/>
-      <c r="F515" s="11"/>
+      <c r="A515" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B515" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C515" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D515" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E515" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="F515" s="9">
+        <v>46227</v>
+      </c>
       <c r="G515" s="12"/>
     </row>
     <row r="516" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A516" s="11"/>
-      <c r="B516" s="11"/>
-      <c r="C516" s="11"/>
-      <c r="D516" s="11"/>
-      <c r="E516" s="11"/>
-      <c r="F516" s="11"/>
+      <c r="A516" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B516" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C516" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D516" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E516" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="F516" s="9">
+        <v>46227</v>
+      </c>
       <c r="G516" s="12"/>
     </row>
     <row r="517" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A517" s="11"/>
-      <c r="B517" s="11"/>
-      <c r="C517" s="11"/>
-      <c r="D517" s="11"/>
-      <c r="E517" s="11"/>
-      <c r="F517" s="11"/>
+      <c r="A517" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B517" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C517" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D517" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E517" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="F517" s="9">
+        <v>46227</v>
+      </c>
       <c r="G517" s="12"/>
     </row>
     <row r="518" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A518" s="11"/>
-      <c r="B518" s="11"/>
-      <c r="C518" s="11"/>
-      <c r="D518" s="11"/>
-      <c r="E518" s="11"/>
-      <c r="F518" s="11"/>
+      <c r="A518" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B518" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C518" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D518" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E518" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="F518" s="9">
+        <v>46227</v>
+      </c>
       <c r="G518" s="12"/>
     </row>
     <row r="519" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A519" s="11"/>
-      <c r="B519" s="11"/>
-      <c r="C519" s="11"/>
-      <c r="D519" s="11"/>
-      <c r="E519" s="11"/>
-      <c r="F519" s="11"/>
+      <c r="A519" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B519" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C519" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D519" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E519" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F519" s="9">
+        <v>46227</v>
+      </c>
       <c r="G519" s="12"/>
+    </row>
+    <row r="520" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A520" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B520" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C520" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D520" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E520" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="F520" s="9">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="521" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A521" s="11"/>
+      <c r="B521" s="11"/>
+      <c r="C521" s="11"/>
+      <c r="D521" s="11"/>
+      <c r="E521" s="11"/>
+      <c r="F521" s="11"/>
+    </row>
+    <row r="522" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A522" s="11"/>
+      <c r="B522" s="11"/>
+      <c r="C522" s="11"/>
+      <c r="D522" s="11"/>
+      <c r="E522" s="11"/>
+      <c r="F522" s="11"/>
+    </row>
+    <row r="523" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A523" s="11"/>
+      <c r="B523" s="11"/>
+      <c r="C523" s="11"/>
+      <c r="D523" s="11"/>
+      <c r="E523" s="11"/>
+      <c r="F523" s="11"/>
+    </row>
+    <row r="524" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A524" s="11"/>
+      <c r="B524" s="11"/>
+      <c r="C524" s="11"/>
+      <c r="D524" s="11"/>
+      <c r="E524" s="11"/>
+      <c r="F524" s="11"/>
+    </row>
+    <row r="525" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A525" s="11"/>
+      <c r="B525" s="11"/>
+      <c r="C525" s="11"/>
+      <c r="D525" s="11"/>
+      <c r="E525" s="11"/>
+      <c r="F525" s="11"/>
+    </row>
+    <row r="526" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A526" s="11"/>
+      <c r="B526" s="11"/>
+      <c r="C526" s="11"/>
+      <c r="D526" s="11"/>
+      <c r="E526" s="11"/>
+      <c r="F526" s="11"/>
+    </row>
+    <row r="527" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A527" s="11"/>
+      <c r="B527" s="11"/>
+      <c r="C527" s="11"/>
+      <c r="D527" s="11"/>
+      <c r="E527" s="11"/>
+      <c r="F527" s="11"/>
+    </row>
+    <row r="528" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A528" s="11"/>
+      <c r="B528" s="11"/>
+      <c r="C528" s="11"/>
+      <c r="D528" s="11"/>
+      <c r="E528" s="11"/>
+      <c r="F528" s="11"/>
+    </row>
+    <row r="529" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A529" s="11"/>
+      <c r="B529" s="11"/>
+      <c r="C529" s="11"/>
+      <c r="D529" s="11"/>
+      <c r="E529" s="11"/>
+      <c r="F529" s="11"/>
+    </row>
+    <row r="530" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A530" s="11"/>
+      <c r="B530" s="11"/>
+      <c r="C530" s="11"/>
+      <c r="D530" s="11"/>
+      <c r="E530" s="11"/>
+      <c r="F530" s="11"/>
+    </row>
+    <row r="531" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A531" s="11"/>
+      <c r="B531" s="11"/>
+      <c r="C531" s="11"/>
+      <c r="D531" s="11"/>
+      <c r="E531" s="11"/>
+      <c r="F531" s="11"/>
+    </row>
+    <row r="532" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A532" s="11"/>
+      <c r="B532" s="11"/>
+      <c r="C532" s="11"/>
+      <c r="D532" s="11"/>
+      <c r="E532" s="11"/>
+      <c r="F532" s="11"/>
+    </row>
+    <row r="533" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A533" s="11"/>
+      <c r="B533" s="11"/>
+      <c r="C533" s="11"/>
+      <c r="D533" s="11"/>
+      <c r="E533" s="11"/>
+      <c r="F533" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
BLAST Premier 2026 Seoul Stage 1
</commit_message>
<xml_diff>
--- a/file/history.xlsx
+++ b/file/history.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/faa3f9bfbb5dc780/Documentos/GitHub/ck-tools/file/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="310" documentId="13_ncr:1_{AB7ADBC0-0AFC-4EB5-BDC6-F57936754D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EA92924-92A5-49A4-93CE-EF44D84367BC}"/>
+  <xr:revisionPtr revIDLastSave="563" documentId="13_ncr:1_{AB7ADBC0-0AFC-4EB5-BDC6-F57936754D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{875A5B4F-0713-4E80-888F-0BBE7E743135}"/>
   <bookViews>
-    <workbookView xWindow="3195" yWindow="1785" windowWidth="23250" windowHeight="12450" xr2:uid="{39BF18F1-6CA4-42F4-B020-2D59954264FB}"/>
+    <workbookView xWindow="2520" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{39BF18F1-6CA4-42F4-B020-2D59954264FB}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2601" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2786" uniqueCount="268">
   <si>
     <t>Team 1</t>
   </si>
@@ -834,6 +834,12 @@
   </si>
   <si>
     <t>Winamax Spanish Cirtuit 2082</t>
+  </si>
+  <si>
+    <t>BLAST Premier 2026 Seoul</t>
+  </si>
+  <si>
+    <t>Lux Tenebris</t>
   </si>
 </sst>
 </file>
@@ -957,10 +963,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1280,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECD49EDF-97AD-42E2-9203-75390A90C7F2}">
-  <dimension ref="A1:H533"/>
+  <dimension ref="A1:H606"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" style="1" customWidth="1"/>
@@ -11379,43 +11381,43 @@
       <c r="G502" s="12"/>
     </row>
     <row r="503" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A503" s="4" t="s">
+      <c r="A503" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="B503" s="4" t="s">
+      <c r="B503" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="C503" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D503" s="4" t="s">
+      <c r="C503" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D503" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="E503" s="4" t="s">
+      <c r="E503" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="F503" s="9">
+      <c r="F503" s="8">
         <v>46225</v>
       </c>
       <c r="G503" s="12"/>
     </row>
     <row r="504" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A504" s="4" t="s">
+      <c r="A504" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="B504" s="4" t="s">
+      <c r="B504" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="C504" s="4" t="s">
+      <c r="C504" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="D504" s="4" t="s">
+      <c r="D504" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="E504" s="4" t="s">
+      <c r="E504" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="F504" s="9">
+      <c r="F504" s="8">
         <v>46225</v>
       </c>
       <c r="G504" s="12"/>
@@ -11484,43 +11486,43 @@
       <c r="G507" s="12"/>
     </row>
     <row r="508" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A508" s="4" t="s">
+      <c r="A508" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="B508" s="4" t="s">
+      <c r="B508" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C508" s="4" t="s">
+      <c r="C508" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D508" s="4" t="s">
+      <c r="D508" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="E508" s="4" t="s">
+      <c r="E508" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="F508" s="9">
+      <c r="F508" s="8">
         <v>46226</v>
       </c>
       <c r="G508" s="12"/>
     </row>
     <row r="509" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A509" s="4" t="s">
+      <c r="A509" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="B509" s="4" t="s">
+      <c r="B509" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C509" s="4" t="s">
+      <c r="C509" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D509" s="4" t="s">
+      <c r="D509" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E509" s="4" t="s">
+      <c r="E509" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="F509" s="9">
+      <c r="F509" s="8">
         <v>46226</v>
       </c>
       <c r="G509" s="12"/>
@@ -11568,64 +11570,64 @@
       <c r="G511" s="12"/>
     </row>
     <row r="512" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A512" s="4" t="s">
+      <c r="A512" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="B512" s="4" t="s">
+      <c r="B512" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="C512" s="4" t="s">
+      <c r="C512" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D512" s="4" t="s">
+      <c r="D512" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E512" s="4" t="s">
+      <c r="E512" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="F512" s="9">
+      <c r="F512" s="8">
         <v>46226</v>
       </c>
       <c r="G512" s="12"/>
     </row>
     <row r="513" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A513" s="4" t="s">
+      <c r="A513" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="B513" s="4" t="s">
+      <c r="B513" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="C513" s="4" t="s">
+      <c r="C513" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D513" s="4" t="s">
+      <c r="D513" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="E513" s="4" t="s">
+      <c r="E513" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="F513" s="9">
+      <c r="F513" s="8">
         <v>46226</v>
       </c>
       <c r="G513" s="12"/>
     </row>
     <row r="514" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A514" s="4" t="s">
+      <c r="A514" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="B514" s="4" t="s">
+      <c r="B514" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="C514" s="4" t="s">
+      <c r="C514" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D514" s="4" t="s">
+      <c r="D514" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="E514" s="4" t="s">
+      <c r="E514" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="F514" s="9">
+      <c r="F514" s="8">
         <v>46226</v>
       </c>
       <c r="G514" s="12"/>
@@ -11673,43 +11675,43 @@
       <c r="G516" s="12"/>
     </row>
     <row r="517" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A517" s="4" t="s">
+      <c r="A517" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B517" s="4" t="s">
+      <c r="B517" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C517" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D517" s="4" t="s">
+      <c r="C517" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D517" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E517" s="4" t="s">
+      <c r="E517" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="F517" s="9">
+      <c r="F517" s="8">
         <v>46227</v>
       </c>
       <c r="G517" s="12"/>
     </row>
     <row r="518" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A518" s="4" t="s">
+      <c r="A518" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B518" s="4" t="s">
+      <c r="B518" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C518" s="4" t="s">
+      <c r="C518" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D518" s="4" t="s">
+      <c r="D518" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E518" s="4" t="s">
+      <c r="E518" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="F518" s="9">
+      <c r="F518" s="8">
         <v>46227</v>
       </c>
       <c r="G518" s="12"/>
@@ -11756,108 +11758,1136 @@
       </c>
     </row>
     <row r="521" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A521" s="11"/>
-      <c r="B521" s="11"/>
-      <c r="C521" s="11"/>
-      <c r="D521" s="11"/>
-      <c r="E521" s="11"/>
-      <c r="F521" s="11"/>
+      <c r="A521" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B521" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C521" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D521" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E521" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F521" s="8">
+        <v>46235</v>
+      </c>
     </row>
     <row r="522" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A522" s="11"/>
-      <c r="B522" s="11"/>
-      <c r="C522" s="11"/>
-      <c r="D522" s="11"/>
-      <c r="E522" s="11"/>
-      <c r="F522" s="11"/>
+      <c r="A522" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B522" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C522" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D522" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E522" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F522" s="8">
+        <v>46235</v>
+      </c>
     </row>
     <row r="523" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A523" s="11"/>
-      <c r="B523" s="11"/>
-      <c r="C523" s="11"/>
-      <c r="D523" s="11"/>
-      <c r="E523" s="11"/>
-      <c r="F523" s="11"/>
+      <c r="A523" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B523" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C523" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D523" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E523" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F523" s="8">
+        <v>46235</v>
+      </c>
     </row>
     <row r="524" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A524" s="11"/>
-      <c r="B524" s="11"/>
-      <c r="C524" s="11"/>
-      <c r="D524" s="11"/>
-      <c r="E524" s="11"/>
-      <c r="F524" s="11"/>
+      <c r="A524" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B524" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C524" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D524" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E524" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F524" s="9">
+        <v>46235</v>
+      </c>
     </row>
     <row r="525" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A525" s="11"/>
-      <c r="B525" s="11"/>
-      <c r="C525" s="11"/>
-      <c r="D525" s="11"/>
-      <c r="E525" s="11"/>
-      <c r="F525" s="11"/>
+      <c r="A525" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B525" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C525" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D525" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E525" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F525" s="9">
+        <v>46235</v>
+      </c>
     </row>
     <row r="526" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A526" s="11"/>
-      <c r="B526" s="11"/>
-      <c r="C526" s="11"/>
-      <c r="D526" s="11"/>
-      <c r="E526" s="11"/>
-      <c r="F526" s="11"/>
+      <c r="A526" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B526" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C526" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D526" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E526" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F526" s="8">
+        <v>46236</v>
+      </c>
     </row>
     <row r="527" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A527" s="11"/>
-      <c r="B527" s="11"/>
-      <c r="C527" s="11"/>
-      <c r="D527" s="11"/>
-      <c r="E527" s="11"/>
-      <c r="F527" s="11"/>
+      <c r="A527" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B527" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C527" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D527" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E527" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F527" s="8">
+        <v>46236</v>
+      </c>
     </row>
     <row r="528" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A528" s="11"/>
-      <c r="B528" s="11"/>
-      <c r="C528" s="11"/>
-      <c r="D528" s="11"/>
-      <c r="E528" s="11"/>
-      <c r="F528" s="11"/>
+      <c r="A528" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B528" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C528" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D528" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E528" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F528" s="8">
+        <v>46236</v>
+      </c>
     </row>
     <row r="529" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A529" s="11"/>
-      <c r="B529" s="11"/>
-      <c r="C529" s="11"/>
-      <c r="D529" s="11"/>
-      <c r="E529" s="11"/>
-      <c r="F529" s="11"/>
+      <c r="A529" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B529" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C529" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D529" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E529" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F529" s="9">
+        <v>46236</v>
+      </c>
     </row>
     <row r="530" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A530" s="11"/>
-      <c r="B530" s="11"/>
-      <c r="C530" s="11"/>
-      <c r="D530" s="11"/>
-      <c r="E530" s="11"/>
-      <c r="F530" s="11"/>
+      <c r="A530" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B530" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C530" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D530" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E530" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F530" s="9">
+        <v>46236</v>
+      </c>
     </row>
     <row r="531" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A531" s="11"/>
-      <c r="B531" s="11"/>
-      <c r="C531" s="11"/>
-      <c r="D531" s="11"/>
-      <c r="E531" s="11"/>
-      <c r="F531" s="11"/>
+      <c r="A531" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B531" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C531" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D531" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E531" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F531" s="8">
+        <v>46237</v>
+      </c>
     </row>
     <row r="532" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A532" s="11"/>
-      <c r="B532" s="11"/>
-      <c r="C532" s="11"/>
-      <c r="D532" s="11"/>
-      <c r="E532" s="11"/>
-      <c r="F532" s="11"/>
+      <c r="A532" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B532" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C532" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D532" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E532" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F532" s="8">
+        <v>46237</v>
+      </c>
     </row>
     <row r="533" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A533" s="11"/>
-      <c r="B533" s="11"/>
-      <c r="C533" s="11"/>
-      <c r="D533" s="11"/>
-      <c r="E533" s="11"/>
-      <c r="F533" s="11"/>
+      <c r="A533" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B533" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C533" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D533" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E533" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F533" s="9">
+        <v>46237</v>
+      </c>
+    </row>
+    <row r="534" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A534" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B534" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C534" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D534" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E534" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F534" s="9">
+        <v>46237</v>
+      </c>
+    </row>
+    <row r="535" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A535" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B535" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C535" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D535" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E535" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F535" s="8">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="536" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A536" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B536" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C536" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D536" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E536" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F536" s="8">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="537" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A537" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B537" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C537" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D537" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E537" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F537" s="9">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="538" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A538" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B538" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C538" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D538" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E538" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F538" s="9">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="539" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A539" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B539" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C539" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D539" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E539" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F539" s="9">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="540" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A540" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B540" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C540" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D540" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E540" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F540" s="8">
+        <v>46239</v>
+      </c>
+    </row>
+    <row r="541" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A541" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B541" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C541" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D541" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E541" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F541" s="8">
+        <v>46239</v>
+      </c>
+    </row>
+    <row r="542" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A542" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B542" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C542" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D542" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E542" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F542" s="9">
+        <v>46239</v>
+      </c>
+    </row>
+    <row r="543" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A543" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B543" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C543" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D543" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E543" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F543" s="9">
+        <v>46239</v>
+      </c>
+    </row>
+    <row r="544" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A544" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B544" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C544" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D544" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E544" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F544" s="9">
+        <v>46239</v>
+      </c>
+    </row>
+    <row r="545" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A545" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B545" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C545" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D545" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E545" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F545" s="8">
+        <v>46240</v>
+      </c>
+    </row>
+    <row r="546" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A546" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B546" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C546" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D546" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E546" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F546" s="8">
+        <v>46240</v>
+      </c>
+    </row>
+    <row r="547" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A547" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B547" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C547" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D547" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E547" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F547" s="9">
+        <v>46240</v>
+      </c>
+    </row>
+    <row r="548" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A548" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B548" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C548" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D548" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="E548" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F548" s="9">
+        <v>46240</v>
+      </c>
+    </row>
+    <row r="549" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A549" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B549" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C549" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D549" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E549" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F549" s="9">
+        <v>46240</v>
+      </c>
+    </row>
+    <row r="550" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A550" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B550" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C550" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D550" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E550" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F550" s="8">
+        <v>46241</v>
+      </c>
+    </row>
+    <row r="551" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A551" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B551" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C551" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D551" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E551" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F551" s="8">
+        <v>46241</v>
+      </c>
+    </row>
+    <row r="552" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A552" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B552" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C552" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D552" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E552" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F552" s="9">
+        <v>46241</v>
+      </c>
+    </row>
+    <row r="553" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A553" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B553" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C553" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D553" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E553" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F553" s="9">
+        <v>46241</v>
+      </c>
+    </row>
+    <row r="554" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A554" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B554" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="C554" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D554" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="E554" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F554" s="8">
+        <v>46242</v>
+      </c>
+    </row>
+    <row r="555" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A555" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B555" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="C555" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D555" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E555" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F555" s="8">
+        <v>46242</v>
+      </c>
+    </row>
+    <row r="556" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A556" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B556" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="C556" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D556" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E556" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F556" s="9">
+        <v>46242</v>
+      </c>
+    </row>
+    <row r="557" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A557" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B557" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="C557" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D557" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="E557" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F557" s="9">
+        <v>46242</v>
+      </c>
+    </row>
+    <row r="558" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A558" s="11"/>
+      <c r="B558" s="11"/>
+      <c r="C558" s="11"/>
+      <c r="D558" s="11"/>
+      <c r="E558" s="11"/>
+      <c r="F558" s="11"/>
+    </row>
+    <row r="559" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A559" s="11"/>
+      <c r="B559" s="11"/>
+      <c r="C559" s="11"/>
+      <c r="D559" s="11"/>
+      <c r="E559" s="11"/>
+      <c r="F559" s="11"/>
+    </row>
+    <row r="560" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A560" s="11"/>
+      <c r="B560" s="11"/>
+      <c r="C560" s="11"/>
+      <c r="D560" s="11"/>
+      <c r="E560" s="11"/>
+      <c r="F560" s="11"/>
+    </row>
+    <row r="561" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A561" s="11"/>
+      <c r="B561" s="11"/>
+      <c r="C561" s="11"/>
+      <c r="D561" s="11"/>
+      <c r="E561" s="11"/>
+      <c r="F561" s="11"/>
+    </row>
+    <row r="562" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A562" s="11"/>
+      <c r="B562" s="11"/>
+      <c r="C562" s="11"/>
+      <c r="D562" s="11"/>
+      <c r="E562" s="11"/>
+      <c r="F562" s="11"/>
+    </row>
+    <row r="563" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A563" s="11"/>
+      <c r="B563" s="11"/>
+      <c r="C563" s="11"/>
+      <c r="D563" s="11"/>
+      <c r="E563" s="11"/>
+      <c r="F563" s="11"/>
+    </row>
+    <row r="564" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A564" s="11"/>
+      <c r="B564" s="11"/>
+      <c r="C564" s="11"/>
+      <c r="D564" s="11"/>
+      <c r="E564" s="11"/>
+      <c r="F564" s="11"/>
+    </row>
+    <row r="565" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A565" s="11"/>
+      <c r="B565" s="11"/>
+      <c r="C565" s="11"/>
+      <c r="D565" s="11"/>
+      <c r="E565" s="11"/>
+      <c r="F565" s="11"/>
+    </row>
+    <row r="566" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A566" s="11"/>
+      <c r="B566" s="11"/>
+      <c r="C566" s="11"/>
+      <c r="D566" s="11"/>
+      <c r="E566" s="11"/>
+      <c r="F566" s="11"/>
+    </row>
+    <row r="567" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A567" s="11"/>
+      <c r="B567" s="11"/>
+      <c r="C567" s="11"/>
+      <c r="D567" s="11"/>
+      <c r="E567" s="11"/>
+      <c r="F567" s="11"/>
+    </row>
+    <row r="568" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A568" s="11"/>
+      <c r="B568" s="11"/>
+      <c r="C568" s="11"/>
+      <c r="D568" s="11"/>
+      <c r="E568" s="11"/>
+      <c r="F568" s="11"/>
+    </row>
+    <row r="569" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A569" s="11"/>
+      <c r="B569" s="11"/>
+      <c r="C569" s="11"/>
+      <c r="D569" s="11"/>
+      <c r="E569" s="11"/>
+      <c r="F569" s="11"/>
+    </row>
+    <row r="570" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A570" s="11"/>
+      <c r="B570" s="11"/>
+      <c r="C570" s="11"/>
+      <c r="D570" s="11"/>
+      <c r="E570" s="11"/>
+      <c r="F570" s="11"/>
+    </row>
+    <row r="571" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A571" s="11"/>
+      <c r="B571" s="11"/>
+      <c r="C571" s="11"/>
+      <c r="D571" s="11"/>
+      <c r="E571" s="11"/>
+      <c r="F571" s="11"/>
+    </row>
+    <row r="572" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A572" s="11"/>
+      <c r="B572" s="11"/>
+      <c r="C572" s="11"/>
+      <c r="D572" s="11"/>
+      <c r="E572" s="11"/>
+      <c r="F572" s="11"/>
+    </row>
+    <row r="573" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A573" s="11"/>
+      <c r="B573" s="11"/>
+      <c r="C573" s="11"/>
+      <c r="D573" s="11"/>
+      <c r="E573" s="11"/>
+      <c r="F573" s="11"/>
+    </row>
+    <row r="574" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A574" s="11"/>
+      <c r="B574" s="11"/>
+      <c r="C574" s="11"/>
+      <c r="D574" s="11"/>
+      <c r="E574" s="11"/>
+      <c r="F574" s="11"/>
+    </row>
+    <row r="575" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A575" s="11"/>
+      <c r="B575" s="11"/>
+      <c r="C575" s="11"/>
+      <c r="D575" s="11"/>
+      <c r="E575" s="11"/>
+      <c r="F575" s="11"/>
+    </row>
+    <row r="576" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A576" s="11"/>
+      <c r="B576" s="11"/>
+      <c r="C576" s="11"/>
+      <c r="D576" s="11"/>
+      <c r="E576" s="11"/>
+      <c r="F576" s="11"/>
+    </row>
+    <row r="577" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A577" s="11"/>
+      <c r="B577" s="11"/>
+      <c r="C577" s="11"/>
+      <c r="D577" s="11"/>
+      <c r="E577" s="11"/>
+      <c r="F577" s="11"/>
+    </row>
+    <row r="578" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A578" s="11"/>
+      <c r="B578" s="11"/>
+      <c r="C578" s="11"/>
+      <c r="D578" s="11"/>
+      <c r="E578" s="11"/>
+      <c r="F578" s="11"/>
+    </row>
+    <row r="579" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A579" s="11"/>
+      <c r="B579" s="11"/>
+      <c r="C579" s="11"/>
+      <c r="D579" s="11"/>
+      <c r="E579" s="11"/>
+      <c r="F579" s="11"/>
+    </row>
+    <row r="580" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A580" s="11"/>
+      <c r="B580" s="11"/>
+      <c r="C580" s="11"/>
+      <c r="D580" s="11"/>
+      <c r="E580" s="11"/>
+      <c r="F580" s="11"/>
+    </row>
+    <row r="581" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A581" s="11"/>
+      <c r="B581" s="11"/>
+      <c r="C581" s="11"/>
+      <c r="D581" s="11"/>
+      <c r="E581" s="11"/>
+      <c r="F581" s="11"/>
+    </row>
+    <row r="582" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A582" s="11"/>
+      <c r="B582" s="11"/>
+      <c r="C582" s="11"/>
+      <c r="D582" s="11"/>
+      <c r="E582" s="11"/>
+      <c r="F582" s="11"/>
+    </row>
+    <row r="583" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A583" s="11"/>
+      <c r="B583" s="11"/>
+      <c r="C583" s="11"/>
+      <c r="D583" s="11"/>
+      <c r="E583" s="11"/>
+      <c r="F583" s="11"/>
+    </row>
+    <row r="584" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A584" s="11"/>
+      <c r="B584" s="11"/>
+      <c r="C584" s="11"/>
+      <c r="D584" s="11"/>
+      <c r="E584" s="11"/>
+      <c r="F584" s="11"/>
+    </row>
+    <row r="585" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A585" s="11"/>
+      <c r="B585" s="11"/>
+      <c r="C585" s="11"/>
+      <c r="D585" s="11"/>
+      <c r="E585" s="11"/>
+      <c r="F585" s="11"/>
+    </row>
+    <row r="586" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A586" s="11"/>
+      <c r="B586" s="11"/>
+      <c r="C586" s="11"/>
+      <c r="D586" s="11"/>
+      <c r="E586" s="11"/>
+      <c r="F586" s="11"/>
+    </row>
+    <row r="587" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A587" s="11"/>
+      <c r="B587" s="11"/>
+      <c r="C587" s="11"/>
+      <c r="D587" s="11"/>
+      <c r="E587" s="11"/>
+      <c r="F587" s="11"/>
+    </row>
+    <row r="588" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A588" s="11"/>
+      <c r="B588" s="11"/>
+      <c r="C588" s="11"/>
+      <c r="D588" s="11"/>
+      <c r="E588" s="11"/>
+      <c r="F588" s="11"/>
+    </row>
+    <row r="589" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A589" s="11"/>
+      <c r="B589" s="11"/>
+      <c r="C589" s="11"/>
+      <c r="D589" s="11"/>
+      <c r="E589" s="11"/>
+      <c r="F589" s="11"/>
+    </row>
+    <row r="590" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A590" s="11"/>
+      <c r="B590" s="11"/>
+      <c r="C590" s="11"/>
+      <c r="D590" s="11"/>
+      <c r="E590" s="11"/>
+      <c r="F590" s="11"/>
+    </row>
+    <row r="591" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A591" s="11"/>
+      <c r="B591" s="11"/>
+      <c r="C591" s="11"/>
+      <c r="D591" s="11"/>
+      <c r="E591" s="11"/>
+      <c r="F591" s="11"/>
+    </row>
+    <row r="592" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A592" s="11"/>
+      <c r="B592" s="11"/>
+      <c r="C592" s="11"/>
+      <c r="D592" s="11"/>
+      <c r="E592" s="11"/>
+      <c r="F592" s="11"/>
+    </row>
+    <row r="593" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A593" s="11"/>
+      <c r="B593" s="11"/>
+      <c r="C593" s="11"/>
+      <c r="D593" s="11"/>
+      <c r="E593" s="11"/>
+      <c r="F593" s="11"/>
+    </row>
+    <row r="594" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A594" s="11"/>
+      <c r="B594" s="11"/>
+      <c r="C594" s="11"/>
+      <c r="D594" s="11"/>
+      <c r="E594" s="11"/>
+      <c r="F594" s="11"/>
+    </row>
+    <row r="595" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A595" s="11"/>
+      <c r="B595" s="11"/>
+      <c r="C595" s="11"/>
+      <c r="D595" s="11"/>
+      <c r="E595" s="11"/>
+      <c r="F595" s="11"/>
+    </row>
+    <row r="596" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A596" s="11"/>
+      <c r="B596" s="11"/>
+      <c r="C596" s="11"/>
+      <c r="D596" s="11"/>
+      <c r="E596" s="11"/>
+      <c r="F596" s="11"/>
+    </row>
+    <row r="597" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A597" s="11"/>
+      <c r="B597" s="11"/>
+      <c r="C597" s="11"/>
+      <c r="D597" s="11"/>
+      <c r="E597" s="11"/>
+      <c r="F597" s="11"/>
+    </row>
+    <row r="598" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A598" s="11"/>
+      <c r="B598" s="11"/>
+      <c r="C598" s="11"/>
+      <c r="D598" s="11"/>
+      <c r="E598" s="11"/>
+      <c r="F598" s="11"/>
+    </row>
+    <row r="599" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A599" s="11"/>
+      <c r="B599" s="11"/>
+      <c r="C599" s="11"/>
+      <c r="D599" s="11"/>
+      <c r="E599" s="11"/>
+      <c r="F599" s="11"/>
+    </row>
+    <row r="600" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A600" s="11"/>
+      <c r="B600" s="11"/>
+      <c r="C600" s="11"/>
+      <c r="D600" s="11"/>
+      <c r="E600" s="11"/>
+      <c r="F600" s="11"/>
+    </row>
+    <row r="601" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A601" s="11"/>
+      <c r="B601" s="11"/>
+      <c r="C601" s="11"/>
+      <c r="D601" s="11"/>
+      <c r="E601" s="11"/>
+      <c r="F601" s="11"/>
+    </row>
+    <row r="602" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A602" s="11"/>
+      <c r="B602" s="11"/>
+      <c r="C602" s="11"/>
+      <c r="D602" s="11"/>
+      <c r="E602" s="11"/>
+      <c r="F602" s="11"/>
+    </row>
+    <row r="603" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A603" s="11"/>
+      <c r="B603" s="11"/>
+      <c r="C603" s="11"/>
+      <c r="D603" s="11"/>
+      <c r="E603" s="11"/>
+      <c r="F603" s="11"/>
+    </row>
+    <row r="604" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A604" s="11"/>
+      <c r="B604" s="11"/>
+      <c r="C604" s="11"/>
+      <c r="D604" s="11"/>
+      <c r="E604" s="11"/>
+      <c r="F604" s="11"/>
+    </row>
+    <row r="605" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A605" s="11"/>
+      <c r="B605" s="11"/>
+      <c r="C605" s="11"/>
+      <c r="D605" s="11"/>
+      <c r="E605" s="11"/>
+      <c r="F605" s="11"/>
+    </row>
+    <row r="606" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A606" s="11"/>
+      <c r="B606" s="11"/>
+      <c r="C606" s="11"/>
+      <c r="D606" s="11"/>
+      <c r="E606" s="11"/>
+      <c r="F606" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>